<commit_message>
precision recall and mrr
</commit_message>
<xml_diff>
--- a/mmrag_evaluation_results.xlsx
+++ b/mmrag_evaluation_results.xlsx
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -574,7 +574,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>0.625</v>
+        <v>0.778</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -582,7 +582,7 @@
         </is>
       </c>
       <c r="I2" t="n">
-        <v>0.7120616436004639</v>
+        <v>0.7160155773162842</v>
       </c>
       <c r="J2" t="n">
         <v>1</v>
@@ -595,10 +595,10 @@
 Supporting Evidence:
 - The cardiac silhouette and mediastinum size are within normal limits. [R1]
 - There is no pulmonary edema. [R1]
-- The chest x-ray appears to be normal, which means that there are no visible signs of abnormalities or issues in the image. [R1-IMAGE]
+- The chest x-ray appears to be normal, which means that there are no visible signs of abnormalities or issues in the image. [R2-IMAGE]
 Next Steps / Recommendations:
-- Clinical correlation recommended to assess the patient's overall health and identify any underlying issues that may not be visible on the x-ray. [Rx]
-- Further evaluation may be needed to rule out all possible conditions or diseases. [Rx]</t>
+- Clinical correlation recommended to assess the patient's overall health and identify any underlying concerns. [Rx]
+- Further evaluation may be necessary depending on the patient's symptoms and medical history. [Rx]</t>
         </is>
       </c>
       <c r="M2" t="inlineStr"/>
@@ -612,16 +612,16 @@
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R2" t="n">
         <v>0.633</v>
       </c>
       <c r="S2" t="n">
-        <v>0.7636184930801392</v>
+        <v>0.8260046731948852</v>
       </c>
       <c r="T2" t="n">
-        <v>0.6983092465400695</v>
+        <v>0.7295023365974427</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -666,7 +666,7 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0.5643822550773621</v>
+        <v>0.5441363453865051</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
@@ -683,14 +683,14 @@
       <c r="L3" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- Borderline cardiomegaly and enlarged pulmonary arteries are noted on the chest X-ray. [R1]
+- Borderline cardiomegaly detected. [R1]
 Supporting Evidence:
-- The chest X-ray shows borderline cardiomegaly, which may indicate mild cardiac enlargement. [R1]
-- Enlarged pulmonary arteries are visible on the X-ray, which could be related to various conditions such as pulmonary hypertension or chronic lung disease. [R1]
-- The lungs appear clear on the X-ray, which suggests that there is no obvious lung disease or infection present. [R1]
+- The chest X-ray shows borderline cardiomegaly, which is an enlargement of the heart. [R1]
+- Enlarged pulmonary arteries are also visible on the X-ray. [R1]
+- The lungs appear clear, indicating no visible signs of lung disease. [R1]
 Next Steps / Recommendations:
-- Clinical correlation with the patient's medical history and symptoms is recommended to further evaluate the significance of the borderline cardiomegaly and enlarged pulmonary arteries. [Rx]
-- Further diagnostic testing, such as an echocardiogram or pulmonary function tests, may be necessary to determine the underlying cause of the abnormal findings on the chest X-ray. [Rx]</t>
+- Clinical correlation with the patient's history and symptoms is recommended to further evaluate the significance of the borderline cardiomegaly. [Rx]
+- Further evaluation with echocardiography or other diagnostic tests may be necessary to assess cardiac function and determine the cause of the borderline cardiomegaly. [Rx]</t>
         </is>
       </c>
       <c r="M3" t="inlineStr"/>
@@ -710,10 +710,10 @@
         <v>0.576</v>
       </c>
       <c r="S3" t="n">
-        <v>0.8693146765232086</v>
+        <v>0.7032409036159516</v>
       </c>
       <c r="T3" t="n">
-        <v>0.7226573382616043</v>
+        <v>0.6396204518079758</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -758,7 +758,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0.222</v>
+        <v>0.75</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -766,7 +766,7 @@
         </is>
       </c>
       <c r="I4" t="n">
-        <v>0.5643539428710938</v>
+        <v>0.5670633316040039</v>
       </c>
       <c r="J4" t="n">
         <v>1</v>
@@ -777,13 +777,13 @@
           <t>Diagnosis / Impression:
 - No signs of cardiomegaly or abnormal cardiac silhouette detected on chest X-ray. [R1], [R2]
 Supporting Evidence:
-- The chest x-ray does not show any signs of cardiomegaly or an abnormal cardiac silhouette. [R1-IMAGE]
+- The chest X-ray does not show any signs of cardiomegaly or an abnormal cardiac silhouette. [R1-IMAGE]
+- The heart appears to be within normal size and shape in the image. [R1-IMAGE]
 - The chest X-ray does not show any signs of cardiomegaly or an abnormal cardiac silhouette. [R2-IMAGE]
-- The heart appears to be within normal size and shape in the image. [R1-IMAGE]
-- The absence of cardiomegaly or abnormal cardiac silhouette on chest X-ray is consistent with a normal cardiac silhouette. [R2]
+- The heart appears to be within normal size and shape in the image. [R2-IMAGE]
 Next Steps / Recommendations:
 - Clinical correlation recommended to further evaluate the patient's symptoms and medical history. [Rx]
-- Follow-up imaging if symptoms persist or worsen. [Rx]</t>
+- Follow-up imaging if symptoms persist, but based on current evidence, it is unlikely to show cardiomegaly or abnormal cardiac silhouette. [Rx]</t>
         </is>
       </c>
       <c r="M4" t="inlineStr"/>
@@ -797,16 +797,16 @@
         <v>1</v>
       </c>
       <c r="Q4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
         <v>0.5639999999999999</v>
       </c>
       <c r="S4" t="n">
-        <v>0.5581061828613281</v>
+        <v>0.7701189994812012</v>
       </c>
       <c r="T4" t="n">
-        <v>0.561053091430664</v>
+        <v>0.6670594997406005</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="W4" t="n">
@@ -889,7 +889,7 @@
         <v>1</v>
       </c>
       <c r="Q5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
         <v>0.531</v>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>0.6857281923294067</v>
+        <v>0.691457211971283</v>
       </c>
       <c r="J6" t="n">
         <v>1</v>
@@ -960,15 +960,15 @@
       <c r="L6" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- No pleural effusion visible on the chest X-ray. [R1], [R2]
+- No pleural effusion detected on chest X-ray. [R1]
 Supporting Evidence:
 - The chest x-ray does not show any visible signs of pleural effusion. [R1-IMAGE]
-- The chest X-ray does not show any visible pleural effusion. [R2-IMAGE]
+- The chest x-ray does not show any visible anatomical findings related to pleural effusion. [R2-IMAGE]
 - The cardiomediastinal silhouette and pulmonary vasculature are within normal limits, which is consistent with the absence of pleural effusion. [R1]
 - There is no pneumothorax or pleural effusion, as stated in the radiology report. [R1]
 Next Steps / Recommendations:
 - Clinical correlation recommended to rule out other potential causes of symptoms. [Rx]
-- Follow-up imaging if symptoms persist, but based on current evidence, it is unlikely to show pleural effusion. [Rx]</t>
+- Follow-up imaging if symptoms persist, but based on current evidence, it is unlikely that pleural effusion will be detected. [Rx]</t>
         </is>
       </c>
       <c r="M6" t="inlineStr"/>
@@ -982,16 +982,16 @@
         <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6" t="n">
         <v>0.644</v>
       </c>
       <c r="S6" t="n">
-        <v>0.816918457698822</v>
+        <v>0.8186371635913848</v>
       </c>
       <c r="T6" t="n">
-        <v>0.7304592288494109</v>
+        <v>0.7313185817956924</v>
       </c>
       <c r="U6" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
         <v>1</v>
       </c>
       <c r="Q7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R7" t="n">
         <v>0.599</v>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -1221,7 +1221,7 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1229,7 +1229,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>0.8089767098426819</v>
+        <v>0.7059441804885864</v>
       </c>
       <c r="J9" t="n">
         <v>1</v>
@@ -1241,11 +1241,11 @@
 - No significant pathologies detected above threshold. [R1]
 Supporting Evidence:
 - The heart, pulmonary structures, and mediastinum are within normal limits. [R1]
-- No pleural effusion or pneumothorax is present. [R1]
-- No focal air space opacity to suggest a pneumonia. [R1]
+- There is no pleural effusion or pneumothorax. [R1]
+- The chest X-ray shows no focal air space opacity to suggest a pneumonia. [R1]
 Next Steps / Recommendations:
-- Clinical correlation recommended to further evaluate the patient's symptoms and history of mitral valve prolapse. [Rx]
-- Follow-up imaging if symptoms persist, but based on the current evidence, no immediate indication for further imaging. [Rx]</t>
+- Clinical correlation recommended to further evaluate the patient's symptoms and history. [Rx]
+- Follow-up imaging if symptoms persist, but no immediate indication for further imaging based on current findings. [Rx]</t>
         </is>
       </c>
       <c r="M9" t="inlineStr"/>
@@ -1259,16 +1259,16 @@
         <v>1</v>
       </c>
       <c r="Q9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R9" t="n">
         <v>0.5649999999999999</v>
       </c>
       <c r="S9" t="n">
-        <v>0.9426930129528045</v>
+        <v>0.8317832541465761</v>
       </c>
       <c r="T9" t="n">
-        <v>0.7538465064764022</v>
+        <v>0.6983916270732879</v>
       </c>
       <c r="U9" t="inlineStr">
         <is>
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="I10" t="n">
-        <v>0.60411536693573</v>
+        <v>0.6633126735687256</v>
       </c>
       <c r="J10" t="n">
         <v>1</v>
@@ -1330,13 +1330,14 @@
       <c r="L10" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- No signs of heart enlargement detected on chest X-ray. [R1], [R2]
+- No heart enlargement detected. [R1-IMAGE], [R2-IMAGE]
 Supporting Evidence:
-- The cardiac silhouette is not enlarged on the chest X-ray. [R1]
+- The cardiac silhouette is not enlarged. [R1]
 - The chest X-ray does not show any signs of heart enlargement. [R1-IMAGE], [R2-IMAGE]
+- There is no consolidation, pleural effusion, or pneumothorax, which can sometimes be associated with heart enlargement. [R1]
 Next Steps / Recommendations:
-- Clinical correlation recommended to further evaluate the patient's symptoms. [Rx]
-- Follow-up imaging if symptoms persist, but no immediate indication for further imaging based on current chest X-ray findings. [Rx]</t>
+- Clinical correlation recommended to assess the patient's overall health and identify any potential issues that may not be visible on the X-ray. [Rx]
+- Further evaluation may be needed to assess the patient's symptoms and determine the cause of chest pain. [Rx]</t>
         </is>
       </c>
       <c r="M10" t="inlineStr"/>
@@ -1350,16 +1351,16 @@
         <v>1</v>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R10" t="n">
         <v>0.594</v>
       </c>
       <c r="S10" t="n">
-        <v>0.8812346100807189</v>
+        <v>0.8989938020706176</v>
       </c>
       <c r="T10" t="n">
-        <v>0.7376173050403594</v>
+        <v>0.7464969010353089</v>
       </c>
       <c r="U10" t="inlineStr">
         <is>
@@ -1395,7 +1396,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E11" t="n">
         <v>1</v>
@@ -1404,7 +1405,7 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0.636</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1412,7 +1413,7 @@
         </is>
       </c>
       <c r="I11" t="n">
-        <v>0.6806971430778503</v>
+        <v>0.6991814970970154</v>
       </c>
       <c r="J11" t="n">
         <v>1</v>
@@ -1423,11 +1424,11 @@
           <t>Diagnosis / Impression:
 - The lung fields appear to be clear on the chest X-ray. [R1-IMAGE]
 Supporting Evidence:
-- The lungs are normally inflated without evidence of focal airspace disease, pleural effusion, or pneumothorax. [R1]
+- The lung fields are normally inflated without evidence of focal airspace disease, pleural effusion, or pneumothorax. [R1]
 - The lung fields appear to be clear on the chest x-ray. [R1-IMAGE]
-- The lung fields appear to be clear on the chest x-ray. [R2-IMAGE]
+- The chest x-ray appears to be normal, which means that there are no visible signs of abnormalities or issues in the lung fields. [R2-IMAGE]
 Next Steps / Recommendations:
-- Clinical correlation recommended to assess the patient's overall health and identify any potential underlying concerns. [Rx]
+- Clinical correlation recommended to assess the patient's overall health and identify any underlying issues that may not be visible on the x-ray. [Rx]
 - Further evaluation may be needed depending on the patient's clinical history and symptoms. [Rx]</t>
         </is>
       </c>
@@ -1442,16 +1443,16 @@
         <v>1</v>
       </c>
       <c r="Q11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R11" t="n">
         <v>0.622</v>
       </c>
       <c r="S11" t="n">
-        <v>0.9042091429233551</v>
+        <v>0.7641544491291046</v>
       </c>
       <c r="T11" t="n">
-        <v>0.7631045714616775</v>
+        <v>0.6930772245645522</v>
       </c>
       <c r="U11" t="inlineStr">
         <is>
@@ -1487,7 +1488,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E12" t="n">
         <v>1</v>
@@ -1504,7 +1505,7 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>0.7782972455024719</v>
+        <v>0.7799336314201355</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
@@ -1520,7 +1521,7 @@
 - No pneumothorax or pleural effusion. [R1]
 - No acute osseous findings. [R1]
 Next Steps / Recommendations:
-- Clinical correlation recommended to assess the patient's overall health and identify any potential concerns. [Rx]
+- Clinical correlation recommended to assess the patient's overall health and identify any underlying concerns. [Rx]
 - Further evaluation may be needed if symptoms persist. [Rx]</t>
         </is>
       </c>
@@ -1535,16 +1536,16 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R12" t="n">
         <v>0.617</v>
       </c>
       <c r="S12" t="n">
-        <v>0.8134891736507415</v>
+        <v>0.8139800894260406</v>
       </c>
       <c r="T12" t="n">
-        <v>0.7152445868253707</v>
+        <v>0.7154900447130204</v>
       </c>
       <c r="U12" t="inlineStr">
         <is>
@@ -1580,7 +1581,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E13" t="n">
         <v>1</v>
@@ -1589,7 +1590,7 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>0.75</v>
+        <v>0.875</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1597,7 +1598,7 @@
         </is>
       </c>
       <c r="I13" t="n">
-        <v>0.820636510848999</v>
+        <v>0.8339194059371948</v>
       </c>
       <c r="J13" t="n">
         <v>1</v>
@@ -1606,7 +1607,7 @@
       <c r="L13" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- No significant abnormal findings detected on the chest X-ray. [R1]
+- No abnormal findings detected on the chest X-ray. [R1]
 Supporting Evidence:
 - Lungs are clear bilaterally. [R1]
 - Cardiac and mediastinal silhouettes are normal. [R1]
@@ -1615,7 +1616,7 @@
 - No acute bony abnormality. [R1]
 Next Steps / Recommendations:
 - Clinical correlation recommended to rule out conditions not visible on chest X-ray. [Rx]
-- Follow-up imaging if symptoms persist or clinical history suggests underlying pathology. [Rx]</t>
+- Follow-up imaging if symptoms persist or clinical history suggests underlying condition. [Rx]</t>
         </is>
       </c>
       <c r="M13" t="inlineStr"/>
@@ -1629,16 +1630,16 @@
         <v>1</v>
       </c>
       <c r="Q13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R13" t="n">
         <v>0.659</v>
       </c>
       <c r="S13" t="n">
-        <v>0.8461909532546998</v>
+        <v>0.9001758217811584</v>
       </c>
       <c r="T13" t="n">
-        <v>0.7525954766273499</v>
+        <v>0.7795879108905792</v>
       </c>
       <c r="U13" t="inlineStr">
         <is>
@@ -1674,7 +1675,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E14" t="n">
         <v>1</v>
@@ -1683,7 +1684,7 @@
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>0.429</v>
+        <v>0.3</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1691,7 +1692,7 @@
         </is>
       </c>
       <c r="I14" t="n">
-        <v>0.8997962474822998</v>
+        <v>0.8635129332542419</v>
       </c>
       <c r="J14" t="n">
         <v>1</v>
@@ -1700,15 +1701,15 @@
       <c r="L14" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- The chest X-ray does not show any signs of cardiomegaly or an abnormal cardiac silhouette. [R1-IMAGE], [R2-IMAGE]
+- No cardiomegaly or abnormal cardiac silhouette detected. [R1-IMAGE], [R2-IMAGE]
 Supporting Evidence:
-- The cardiac silhouette is borderline enlarged on the chest radiograph. [R1]
-- Mediastinal contours are within normal limits on the chest radiograph. [R1]
-- The chest X-ray does not show any large pleural effusion or pneumothorax. [R1]
-- The heart appears to be within normal size and shape on the image. [R2-IMAGE]
+- The chest x-ray does not show any signs of cardiomegaly. [R1-IMAGE]
+- The mediastinal contours are within normal limits. [R1]
+- There is no large pleural effusion or pneumothorax. [R1]
+- The cardiac silhouette is borderline enlarged, but this is not a definitive indicator of cardiomegaly. [R1]
 Next Steps / Recommendations:
-- Clinical correlation recommended to further evaluate the borderline enlarged cardiac silhouette. [Rx]
-- Follow-up imaging if symptoms persist, considering the borderline enlarged cardiac silhouette. [Rx]</t>
+- Clinical correlation recommended to further evaluate the patient's symptoms and medical history. [Rx]
+- Follow-up imaging if symptoms persist or worsen. [Rx]</t>
         </is>
       </c>
       <c r="M14" t="inlineStr"/>
@@ -1722,16 +1723,16 @@
         <v>1</v>
       </c>
       <c r="Q14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R14" t="n">
         <v>0.726</v>
       </c>
       <c r="S14" t="n">
-        <v>0.74153887424469</v>
+        <v>0.6790538799762725</v>
       </c>
       <c r="T14" t="n">
-        <v>0.733769437122345</v>
+        <v>0.7025269399881362</v>
       </c>
       <c r="U14" t="inlineStr">
         <is>
@@ -1740,7 +1741,7 @@
       </c>
       <c r="V14" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>RETRY</t>
         </is>
       </c>
       <c r="W14" t="n">
@@ -1776,7 +1777,7 @@
         <v>1</v>
       </c>
       <c r="G15" t="n">
-        <v>0.714</v>
+        <v>0.75</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1784,7 +1785,7 @@
         </is>
       </c>
       <c r="I15" t="n">
-        <v>0.7411871552467346</v>
+        <v>0.8714293837547302</v>
       </c>
       <c r="J15" t="n">
         <v>1</v>
@@ -1795,12 +1796,13 @@
           <t>Diagnosis / Impression:
 - No signs of pulmonary congestion or edema detected on the chest X-ray. [R1], [R2]
 Supporting Evidence:
-- The chest x-ray shows no focal alveolar consolidation, no definite pleural effusion seen. [R1]
-- No typical findings of pulmonary edema are present on the chest x-ray. [R1]
-- The chest x-ray does not show any signs of pulmonary congestion or edema. [R2-IMAGE]
+- The chest x-ray shows heart size within normal limits, stable mediastinal and hilar contours. [R1]
+- Mild hyperinflation appears similar to prior, with no focal alveolar consolidation or definite pleural effusion seen. [R1]
+- Scattered chronic appearing irregular interstitial markings are present, but no typical findings of pulmonary edema are observed. [R1]
+- The chest x-ray does not show any signs of pulmonary congestion or edema. [R1-IMAGE], [R2-IMAGE]
 Next Steps / Recommendations:
-- Clinical correlation recommended to determine the overall health status of the patient. [Rx]
-- Further evaluation by a healthcare professional is necessary to assess the patient's condition. [Rx]</t>
+- Clinical correlation recommended to further evaluate the patient's symptoms and medical history. [Rx]
+- Follow-up imaging if symptoms persist, but based on the current chest X-ray findings, it does not appear necessary. [Rx]</t>
         </is>
       </c>
       <c r="M15" t="inlineStr"/>
@@ -1814,16 +1816,16 @@
         <v>1</v>
       </c>
       <c r="Q15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R15" t="n">
         <v>0.67</v>
       </c>
       <c r="S15" t="n">
-        <v>0.8079561465740204</v>
+        <v>0.8614288151264191</v>
       </c>
       <c r="T15" t="n">
-        <v>0.7389780732870102</v>
+        <v>0.7657144075632096</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
@@ -1868,7 +1870,7 @@
         <v>1</v>
       </c>
       <c r="G16" t="n">
-        <v>0.8</v>
+        <v>0.429</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1876,7 +1878,7 @@
         </is>
       </c>
       <c r="I16" t="n">
-        <v>0.7225977778434753</v>
+        <v>0.5505229830741882</v>
       </c>
       <c r="J16" t="n">
         <v>1</v>
@@ -1885,15 +1887,15 @@
       <c r="L16" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- No pleural effusion visible on the chest X-ray. [R1], [R2]
+- No visible pleural effusion detected on chest X-ray. [R1-IMAGE], [R2-IMAGE]
 Supporting Evidence:
-- The chest X-ray does not show any visible pleural effusion. [R1-IMAGE]
-- The chest x-ray does not show any visible pleural effusion. [R2-IMAGE]
-- Cardiomediastinal silhouette and pulmonary vasculature are within normal limits, which is consistent with the absence of pleural effusion. [R1]
-- Lungs are clear, further supporting the absence of pleural effusion. [R1]
+- The chest x-ray does not show any visible pleural effusion. [R1-IMAGE]
+- The chest x-ray does not show any visible signs of pleural effusion. [R2-IMAGE]
+- The absence of visible pleural effusion in a chest x-ray does not necessarily rule out the presence of fluid accumulation in the pleural space. [R1-IMAGE]
+- Further diagnostic tests, such as a chest CT scan or ultrasound, may be needed to confirm the presence or absence of pleural effusion. [R1-IMAGE]
 Next Steps / Recommendations:
-- Clinical correlation recommended to assess the cause of dyspnea. [Rx]
-- Follow-up imaging if symptoms persist, but pleural effusion is unlikely given the current findings. [Rx]</t>
+- Clinical correlation recommended to assess the presence of pleural effusion despite negative chest X-ray findings. [Rx]
+- Follow-up imaging with a chest CT scan or ultrasound if symptoms persist or worsen. [Rx]</t>
         </is>
       </c>
       <c r="M16" t="inlineStr"/>
@@ -1907,16 +1909,16 @@
         <v>1</v>
       </c>
       <c r="Q16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R16" t="n">
         <v>0.573</v>
       </c>
       <c r="S16" t="n">
-        <v>0.8367793333530427</v>
+        <v>0.6367568949222565</v>
       </c>
       <c r="T16" t="n">
-        <v>0.7048896666765213</v>
+        <v>0.6048784474611282</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
@@ -1925,7 +1927,7 @@
       </c>
       <c r="V16" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>RETRY</t>
         </is>
       </c>
       <c r="W16" t="n">
@@ -1948,34 +1950,86 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ERROR</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>ragas_failed</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr">
         <is>
-          <t>unsupported operand type(s) for *: 'NoneType' and 'float'</t>
+          <t>Diagnosis / Impression:
+No pathologies detected above threshold on the chest X-ray. [R1]
+Supporting Evidence:
+- The DenseNet CNN algorithm used for pathology detection did not identify any abnormalities above the set threshold. [R1]
+- The absence of pathologies detected by the algorithm suggests that the chest X-ray is likely normal or shows no significant abnormalities. [R2]
+- However, it is essential to note that the absence of findings on a chest X-ray does not rule out the presence of lung consolidation or opacities, especially if they are mild or not severe enough to be detected by the algorithm. [R3]
+Next Steps / Recommendations:
+- Clinical correlation with the patient's symptoms and medical history is recommended to determine the significance of the normal chest X-ray findings. [Rx]
+- If the patient's symptoms persist or worsen, follow-up imaging may be necessary to rule out any underlying conditions. [Rx]</t>
         </is>
       </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr"/>
-      <c r="O17" t="inlineStr"/>
-      <c r="P17" t="inlineStr"/>
-      <c r="Q17" t="inlineStr"/>
-      <c r="R17" t="inlineStr"/>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
-      <c r="V17" t="inlineStr"/>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>3</v>
+      </c>
+      <c r="O17" t="n">
+        <v>2</v>
+      </c>
+      <c r="P17" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>2</v>
+      </c>
+      <c r="R17" t="n">
+        <v>0</v>
+      </c>
+      <c r="S17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="T17" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>FAIL</t>
+        </is>
+      </c>
+      <c r="W17" t="n">
+        <v>0</v>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>XRAY</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -2040,7 +2094,7 @@
         <v>1</v>
       </c>
       <c r="Q18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R18" t="n">
         <v>0.774</v>
@@ -2085,7 +2139,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E19" t="n">
         <v>1</v>
@@ -2094,7 +2148,7 @@
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>0.267</v>
+        <v>0.75</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -2102,7 +2156,7 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>0.6915655136108398</v>
+        <v>0.8006788492202759</v>
       </c>
       <c r="J19" t="n">
         <v>1</v>
@@ -2111,15 +2165,15 @@
       <c r="L19" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- The chest X-ray shows several key findings, including cardiomegaly, bilateral pleural effusions, right-sided pneumothorax, left-sided pneumothorax, bilateral rib fractures, right-sided hemopneumothorax, and left-sided pneumomediastinum. [R1-IMAGE], [R2-IMAGE]
+- No significant pathologies detected above threshold. [R1], [R2]
 Supporting Evidence:
-- Cardiomegaly, which is an enlargement of the heart, is visible on the chest X-ray. [R1-IMAGE]
-- Bilateral pleural effusions, which are abnormal accumulations of fluid in the pleural space surrounding both lungs, are present. [R1-IMAGE]
-- Right-sided pneumothorax, which is a collapsed lung on the right side, is visible on the chest X-ray. [R1-IMAGE]
-- Left-sided pneumothorax, which is a collection of air or gas in the pleural space causing the lung to collapse, is present. [R2-IMAGE]
+- Heart size within normal limits. [R1]
+- No focal alveolar consolidation, no definite pleural effusion seen. [R1]
+- No typical findings of pulmonary edema. [R1]
+- No pneumothorax. [R1]
 Next Steps / Recommendations:
-- Clinical correlation with the patient's symptoms and medical history is recommended to determine the cause of the observed abnormalities. [Rx]
-- Follow-up imaging may be necessary if the patient's symptoms persist or worsen. [Rx]</t>
+- Clinical correlation recommended. [Rx]
+- Insufficient evidence [Rx]</t>
         </is>
       </c>
       <c r="M19" t="inlineStr"/>
@@ -2133,16 +2187,16 @@
         <v>1</v>
       </c>
       <c r="Q19" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="R19" t="n">
         <v>0.612</v>
       </c>
       <c r="S19" t="n">
-        <v>0.614269654083252</v>
+        <v>0.8402036547660828</v>
       </c>
       <c r="T19" t="n">
-        <v>0.6131348270416259</v>
+        <v>0.7261018273830414</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
@@ -2151,7 +2205,7 @@
       </c>
       <c r="V19" t="inlineStr">
         <is>
-          <t>RETRY</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="W19" t="n">
@@ -2178,7 +2232,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E20" t="n">
         <v>1</v>
@@ -2187,7 +2241,7 @@
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>0.75</v>
+        <v>0.444</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2195,7 +2249,7 @@
         </is>
       </c>
       <c r="I20" t="n">
-        <v>0.5309703946113586</v>
+        <v>0.5567283630371094</v>
       </c>
       <c r="J20" t="n">
         <v>1</v>
@@ -2204,15 +2258,15 @@
       <c r="L20" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- No heart enlargement detected on chest X-ray. [R1], [R2]
+- No heart enlargement detected on chest X-ray. [R1-IMAGE], [R2-IMAGE]
 Supporting Evidence:
 - The chest X-ray does not show any signs of heart enlargement. [R1-IMAGE]
-- The chest X-ray does not show any signs of heart enlargement. [R2-IMAGE]
-- Heart size is normal on the X-ray findings. [R1]
-- No signs of heart enlargement were observed on the chest X-ray. [R1]
+- The chest x-ray appears to be normal. [R2-IMAGE]
+- A chest X-ray is a standard tool for assessing heart size, but it may not always detect subtle abnormalities. [R1]
+- Further evaluation may be needed to assess the patient's overall cardiovascular health. [R2]
 Next Steps / Recommendations:
-- Clinical correlation recommended to confirm the absence of heart enlargement. [Rx]
-- Further evaluation with echocardiography or other diagnostic tests may be necessary if symptoms persist. [Rx]</t>
+- Clinical correlation with other diagnostic tests (e.g., ECG, echocardiogram) is recommended to confirm the absence of heart enlargement. [Rx]
+- Follow-up imaging if symptoms persist or if there is a change in clinical status. [Rx]</t>
         </is>
       </c>
       <c r="M20" t="inlineStr"/>
@@ -2226,16 +2280,16 @@
         <v>1</v>
       </c>
       <c r="Q20" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R20" t="n">
         <v>0.605</v>
       </c>
       <c r="S20" t="n">
-        <v>0.7592911183834077</v>
+        <v>0.6446185089111328</v>
       </c>
       <c r="T20" t="n">
-        <v>0.6821455591917038</v>
+        <v>0.6248092544555663</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
@@ -2244,7 +2298,7 @@
       </c>
       <c r="V20" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>RETRY</t>
         </is>
       </c>
       <c r="W20" t="n">
@@ -2271,7 +2325,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E21" t="n">
         <v>1</v>
@@ -2288,7 +2342,7 @@
         </is>
       </c>
       <c r="I21" t="n">
-        <v>0.6488034725189209</v>
+        <v>0.6545675992965698</v>
       </c>
       <c r="J21" t="n">
         <v>1</v>
@@ -2298,14 +2352,13 @@
         <is>
           <t>Diagnosis / Impression:
 - The lung fields appear to be clear on the chest X-ray. [R1-IMAGE]
-- The lung fields appear to be clear on the chest X-ray. [R2-IMAGE]
 Supporting Evidence:
 - The lungs are well expanded and clear. [R1]
+- The lung fields appear to be clear on the chest x-ray. [R1-IMAGE]
 - There are no focal air space opacities. [R1]
-- The lung fields appear to be clear on the chest x-ray. [R1-IMAGE]
 - The lung fields appear to be clear on the chest x-ray. [R2-IMAGE]
 Next Steps / Recommendations:
-- Clinical correlation recommended to determine the patient's overall health status and identify any potential underlying concerns. [Rx]
+- Clinical correlation recommended to rule out underlying conditions. [Rx]
 - Further evaluation may be needed depending on the patient's clinical history and symptoms. [Rx]</t>
         </is>
       </c>
@@ -2320,16 +2373,16 @@
         <v>1</v>
       </c>
       <c r="Q21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R21" t="n">
         <v>0.619</v>
       </c>
       <c r="S21" t="n">
-        <v>0.8946410417556763</v>
+        <v>0.8963702797889709</v>
       </c>
       <c r="T21" t="n">
-        <v>0.7568205208778381</v>
+        <v>0.7576851398944855</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
@@ -2374,7 +2427,7 @@
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>0.667</v>
+        <v>0</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -2382,7 +2435,7 @@
         </is>
       </c>
       <c r="I22" t="n">
-        <v>0.493852436542511</v>
+        <v>0.4528967440128326</v>
       </c>
       <c r="J22" t="n">
         <v>1</v>
@@ -2392,13 +2445,15 @@
         <is>
           <t>Diagnosis / Impression:
 - The chest X-ray appears normal. [R1-IMAGE]
+- The chest X-ray appears to be normal, which means that there are no visible signs of abnormalities or issues in the image. This is consistent with the patient's clinical presentation and the absence of any significant findings on the chest X-ray. [R2-IMAGE]
 Supporting Evidence:
-- The chest x-ray shows no visible signs of abnormalities or issues in the image. [R1-IMAGE]
-- A normal chest x-ray does not necessarily rule out all possible conditions or diseases. [R1-IMAGE]
-- Further evaluation and clinical correlation may be needed to assess the patient's overall health and identify any underlying issues that may not be visible on the x-ray. [R2-IMAGE]
+- The chest x-ray appears to be normal, which means that there are no visible abnormalities or signs of disease in the image. [R1-IMAGE]
+- The chest X-ray appears to be normal, which means that there are no visible signs of abnormalities or issues in the image. [R2-IMAGE]
+- A normal chest x-ray does not necessarily rule out all possible conditions or issues, but it is a reassuring finding that can help guide further evaluation and clinical correlation. [R1-IMAGE]
+- Further evaluation and clinical correlation may be needed to assess the patient's overall health and identify any underlying concerns. [R2-IMAGE]
 Next Steps / Recommendations:
-- Clinical correlation recommended to assess the patient's overall health and identify any underlying issues. [Rx]
-- Further evaluation and tests may be needed depending on the patient's symptoms and clinical history. [Rx]</t>
+- Clinical correlation recommended to assess the patient's overall health and identify any underlying concerns. [Rx]
+- Follow-up imaging if symptoms persist or new symptoms develop. [Rx]</t>
         </is>
       </c>
       <c r="M22" t="inlineStr"/>
@@ -2412,16 +2467,16 @@
         <v>1</v>
       </c>
       <c r="Q22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R22" t="n">
         <v>0.593</v>
       </c>
       <c r="S22" t="n">
-        <v>0.7149557309627532</v>
+        <v>0.4358690232038498</v>
       </c>
       <c r="T22" t="n">
-        <v>0.6539778654813766</v>
+        <v>0.5144345116019249</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
@@ -2430,7 +2485,7 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="W22" t="n">
@@ -2504,7 +2559,7 @@
         <v>1</v>
       </c>
       <c r="Q23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R23" t="n">
         <v>0.637</v>
@@ -2549,7 +2604,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E24" t="n">
         <v>1</v>
@@ -2598,7 +2653,7 @@
         <v>1</v>
       </c>
       <c r="Q24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R24" t="n">
         <v>0.473</v>
@@ -2652,7 +2707,7 @@
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>0.714</v>
+        <v>0.833</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -2660,7 +2715,7 @@
         </is>
       </c>
       <c r="I25" t="n">
-        <v>0.7096673250198364</v>
+        <v>0.5938956737518311</v>
       </c>
       <c r="J25" t="n">
         <v>1</v>
@@ -2672,12 +2727,11 @@
 - No signs of pulmonary congestion or edema detected on the chest X-ray. [R1-IMAGE], [R2-IMAGE]
 Supporting Evidence:
 - The chest x-ray does not show any signs of pulmonary congestion or edema. [R1-IMAGE]
-- The lungs appear to be clear and free of any significant fluid accumulation or other abnormalities in the image. [R2-IMAGE]
-- Cardiomediastinal silhouette is within normal limits of size and appearance, indicating no signs of pulmonary congestion. [R1]
-- Pulmonary vascularity is unremarkable, which is consistent with the absence of pulmonary congestion or edema. [R1]
+- The lungs are expanded and clear of airspace disease. [R1]
+- There is no visible abnormality in the lungs that would indicate fluid accumulation or swelling. [R2-IMAGE]
 Next Steps / Recommendations:
 - Clinical correlation recommended to further evaluate the patient's symptoms of dyspnea. [Rx]
-- Follow-up imaging if symptoms persist, but based on the current chest X-ray findings, it is unlikely to show signs of pulmonary congestion or edema. [Rx]</t>
+- Follow-up imaging if symptoms persist, but based on current evidence, it is unlikely to show signs of pulmonary congestion or edema. [Rx]</t>
         </is>
       </c>
       <c r="M25" t="inlineStr"/>
@@ -2691,16 +2745,16 @@
         <v>1</v>
       </c>
       <c r="Q25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R25" t="n">
         <v>0.55</v>
       </c>
       <c r="S25" t="n">
-        <v>0.7985001975059509</v>
+        <v>0.8113687021255493</v>
       </c>
       <c r="T25" t="n">
-        <v>0.6742500987529755</v>
+        <v>0.6806843510627747</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
@@ -2745,7 +2799,7 @@
         <v>1</v>
       </c>
       <c r="G26" t="n">
-        <v>0.462</v>
+        <v>0</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -2753,7 +2807,7 @@
         </is>
       </c>
       <c r="I26" t="n">
-        <v>0.6392327547073364</v>
+        <v>0.5254111886024475</v>
       </c>
       <c r="J26" t="n">
         <v>1</v>
@@ -2762,14 +2816,14 @@
       <c r="L26" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- Pleural effusion is visible on the chest X-ray. [R1]
+- Pleural effusion is not visible on the chest X-ray, but further imaging techniques such as CT scans may be needed for a more accurate assessment. [R1-IMAGE]
 Supporting Evidence:
-- The chest X-ray shows moderate left pleural effusion and small right pleural effusion. [R1]
-- The lungs are hyperlucent and hyperinflated compatible with emphysema, which may be associated with pleural effusion. [R1]
-- The presence of pleural effusion is confirmed by the pathology detection results, with R1 and R2 showing high confidence in pleural effusion detection. [R1, R2] [R1]
+- The chest x-ray does not show any visible pleural effusion. [R1-IMAGE]
+- A chest x-ray may not always detect subtle or small amounts of pleural effusion. [R1-IMAGE]
+- The chest x-ray does not show any visible pleural effusion. [R2-IMAGE]
 Next Steps / Recommendations:
-- Clinical correlation recommended to assess the cause and severity of the pleural effusion. [Rx]
-- Follow-up imaging if symptoms persist or worsen. [Rx]</t>
+- Clinical correlation recommended to assess the presence of pleural effusion. [Rx]
+- Follow-up imaging with CT scan if symptoms persist or if pleural effusion is suspected. [Rx]</t>
         </is>
       </c>
       <c r="M26" t="inlineStr"/>
@@ -2789,10 +2843,10 @@
         <v>0.599</v>
       </c>
       <c r="S26" t="n">
-        <v>0.6765698264122009</v>
+        <v>0.4576233565807343</v>
       </c>
       <c r="T26" t="n">
-        <v>0.6377849132061004</v>
+        <v>0.5283116782903672</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
@@ -2801,7 +2855,7 @@
       </c>
       <c r="V26" t="inlineStr">
         <is>
-          <t>RETRY</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="W26" t="n">
@@ -2828,7 +2882,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E27" t="n">
         <v>1</v>
@@ -2930,7 +2984,7 @@
         <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>0.714</v>
+        <v>0.857</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -2975,10 +3029,10 @@
         <v>0.5629999999999999</v>
       </c>
       <c r="S28" t="n">
-        <v>0.7969259196281433</v>
+        <v>0.8541259196281433</v>
       </c>
       <c r="T28" t="n">
-        <v>0.6799629598140716</v>
+        <v>0.7085629598140717</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
@@ -3014,7 +3068,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
@@ -3023,7 +3077,7 @@
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>0.714</v>
+        <v>0.333</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -3031,7 +3085,7 @@
         </is>
       </c>
       <c r="I29" t="n">
-        <v>0.7593117952346802</v>
+        <v>0.6758285760879517</v>
       </c>
       <c r="J29" t="n">
         <v>1</v>
@@ -3040,14 +3094,14 @@
       <c r="L29" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- Bilateral patchy pulmonary opacities and pulmonary vascular congestion are noted, with a stable enlarged cardiomediastinal silhouette. [R1]
+- Cardiomegaly and bilateral pleural effusions are present. [R2-IMAGE]
 Supporting Evidence:
-- Interval improvement in left base consolidative opacity is observed. [R1]
-- Pulmonary vascular congestion is again noted. [R1]
-- A stable enlarged cardiomediastinal silhouette is present. [R1]
+- Cardiomegaly is an enlargement of the heart. [R2-IMAGE]
+- Bilateral pleural effusions are abnormal accumulations of fluid in the pleural space surrounding both lungs. [R2-IMAGE]
+- A left-sided pneumothorax is a collection of air or gas in the pleural space that can cause the lung to collapse. [R2-IMAGE]
 Next Steps / Recommendations:
-- Clinical correlation recommended to determine the cause of the observed pulmonary opacities and vascular congestion. [Rx]
-- Further evaluation and consultation with a healthcare professional are necessary to determine the appropriate treatment. [Rx]</t>
+- Clinical correlation recommended to determine the cause of cardiomegaly and pleural effusions. [Rx]
+- Follow-up imaging if symptoms persist to assess for any changes in the patient's condition. [Rx]</t>
         </is>
       </c>
       <c r="M29" t="inlineStr"/>
@@ -3061,16 +3115,16 @@
         <v>1</v>
       </c>
       <c r="Q29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R29" t="n">
         <v>0.533</v>
       </c>
       <c r="S29" t="n">
-        <v>0.8133935385704041</v>
+        <v>0.6359485728263855</v>
       </c>
       <c r="T29" t="n">
-        <v>0.6731967692852021</v>
+        <v>0.5844742864131928</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
@@ -3079,7 +3133,7 @@
       </c>
       <c r="V29" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>RETRY</t>
         </is>
       </c>
       <c r="W29" t="n">
@@ -3106,7 +3160,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="E30" t="n">
         <v>1</v>
@@ -3115,7 +3169,7 @@
         <v>1</v>
       </c>
       <c r="G30" t="n">
-        <v>0.833</v>
+        <v>0</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -3123,7 +3177,7 @@
         </is>
       </c>
       <c r="I30" t="n">
-        <v>0.567784309387207</v>
+        <v>0.4739030599594116</v>
       </c>
       <c r="J30" t="n">
         <v>1</v>
@@ -3132,14 +3186,14 @@
       <c r="L30" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- Insufficient evidence [R1], [R2] to indicate heart enlargement.
+- Insufficient evidence [R1], [R2] to confirm or rule out heart enlargement.
 Supporting Evidence:
 - The chest X-ray does not show any signs of heart enlargement. [R1-IMAGE]
+- The chest X-ray appears to be normal, with no visible abnormalities or issues related to the heart. [R1-IMAGE]
 - The chest X-ray does not show any signs of heart enlargement. [R2-IMAGE]
-- No significant pathologies detected above threshold, including heart enlargement. [R2]
 Next Steps / Recommendations:
-- Clinical correlation recommended to further evaluate symptoms of hypoxia. [Rx]
-- Further diagnostic testing, such as echocardiogram or electrocardiogram, may be necessary to assess heart function. [Rx]</t>
+- Clinical correlation recommended to further evaluate the patient's symptoms and medical history. [Rx]
+- Follow-up imaging if symptoms persist or new symptoms develop. [Rx]</t>
         </is>
       </c>
       <c r="M30" t="inlineStr"/>
@@ -3153,16 +3207,16 @@
         <v>1</v>
       </c>
       <c r="Q30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R30" t="n">
         <v>0.5</v>
       </c>
       <c r="S30" t="n">
-        <v>0.8035352928161621</v>
+        <v>0.4421709179878235</v>
       </c>
       <c r="T30" t="n">
-        <v>0.651767646408081</v>
+        <v>0.4710854589939117</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
@@ -3171,7 +3225,7 @@
       </c>
       <c r="V30" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="W30" t="n">
@@ -3198,7 +3252,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E31" t="n">
         <v>1</v>
@@ -3207,7 +3261,7 @@
         <v>1</v>
       </c>
       <c r="G31" t="n">
-        <v>0.6</v>
+        <v>0.667</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -3215,7 +3269,7 @@
         </is>
       </c>
       <c r="I31" t="n">
-        <v>0.7696354985237122</v>
+        <v>0.7221204042434692</v>
       </c>
       <c r="J31" t="n">
         <v>1</v>
@@ -3226,12 +3280,12 @@
           <t>Diagnosis / Impression:
 - The lung fields appear to be clear on the chest X-ray. [R1-IMAGE]
 Supporting Evidence:
-- Lungs are clear without focal consolidation, effusion, or pneumothorax. [R1]
-- The lung fields appear to be clear on the chest x-ray. [R1-IMAGE]
-- Normal heart size and negative for pneumoperitoneum. [R1]
+- The lungs are clear without focal consolidation, effusion, or pneumothorax. [R1]
+- The chest x-ray appears to be normal, with no visible signs of abnormalities or issues in the lung fields. [R1-IMAGE]
+- The lung fields appear to be clear on the chest x-ray. [R2-IMAGE]
 Next Steps / Recommendations:
 - Clinical correlation recommended to assess the patient's overall health and identify any potential underlying concerns. [Rx]
-- Further evaluation may be needed to rule out all possible conditions or issues. [Rx]</t>
+- Further evaluation may be needed to assess the patient's overall health and identify any underlying conditions that may not be visible on the x-ray. [Rx]</t>
         </is>
       </c>
       <c r="M31" t="inlineStr"/>
@@ -3245,16 +3299,16 @@
         <v>1</v>
       </c>
       <c r="Q31" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R31" t="n">
         <v>0.588</v>
       </c>
       <c r="S31" t="n">
-        <v>0.7708906495571137</v>
+        <v>0.7834361212730407</v>
       </c>
       <c r="T31" t="n">
-        <v>0.6794453247785568</v>
+        <v>0.6857180606365203</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
@@ -3299,7 +3353,7 @@
         <v>1</v>
       </c>
       <c r="G32" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -3307,7 +3361,7 @@
         </is>
       </c>
       <c r="I32" t="n">
-        <v>0.5892553329467773</v>
+        <v>0.5627533793449402</v>
       </c>
       <c r="J32" t="n">
         <v>1</v>
@@ -3318,12 +3372,13 @@
           <t>Diagnosis / Impression:
 - The chest X-ray appears normal. [R1-IMAGE], [R2-IMAGE]
 Supporting Evidence:
-- The chest x-ray shows no visible abnormalities or signs of disease. [R1-IMAGE]
-- The chest x-ray appears to be normal, with no visible signs of issues in the image. [R2-IMAGE]
-- A normal chest x-ray does not necessarily rule out all possible conditions or diseases. [R1-IMAGE], [R2-IMAGE]
+- The chest x-ray shows no visible signs of abnormalities or issues in the image. [R1-IMAGE]
+- The chest X-ray appears to be normal, with no visible abnormalities or signs of disease in the image. [R2-IMAGE]
+- A normal chest x-ray does not necessarily rule out all possible conditions or diseases, and further evaluation and tests may be needed depending on the patient's clinical history and symptoms. [R1-IMAGE]
+- Further evaluation and clinical correlation may be needed to assess the patient's overall health and identify any underlying concerns that may not be apparent on the X-ray. [R2-IMAGE]
 Next Steps / Recommendations:
-- Further evaluation and clinical correlation may be needed to assess the patient's overall health and identify any underlying concerns. [R1-IMAGE], [R2-IMAGE]
-- Clinical correlation is recommended to assess the patient's overall health and identify any underlying issues. [Rx]</t>
+- Clinical correlation recommended to assess the patient's overall health and identify any underlying concerns that may not be apparent on the X-ray. [Rx]
+- Further evaluation and tests may be needed depending on the patient's clinical history and symptoms. [Rx]</t>
         </is>
       </c>
       <c r="M32" t="inlineStr"/>
@@ -3343,10 +3398,10 @@
         <v>0.537</v>
       </c>
       <c r="S32" t="n">
-        <v>0.6767765998840332</v>
+        <v>0.468826013803482</v>
       </c>
       <c r="T32" t="n">
-        <v>0.6068882999420167</v>
+        <v>0.502913006901741</v>
       </c>
       <c r="U32" t="inlineStr">
         <is>
@@ -3355,7 +3410,7 @@
       </c>
       <c r="V32" t="inlineStr">
         <is>
-          <t>RETRY</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="W32" t="n">
@@ -3382,7 +3437,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E33" t="n">
         <v>1</v>
@@ -3430,7 +3485,7 @@
         <v>1</v>
       </c>
       <c r="Q33" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R33" t="n">
         <v>0.662</v>
@@ -3475,7 +3530,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E34" t="n">
         <v>1</v>
@@ -3523,7 +3578,7 @@
         <v>1</v>
       </c>
       <c r="Q34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R34" t="n">
         <v>0.632</v>
@@ -3615,7 +3670,7 @@
         <v>1</v>
       </c>
       <c r="Q35" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R35" t="n">
         <v>0.636</v>
@@ -3669,7 +3724,7 @@
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>0.571</v>
+        <v>0.714</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -3677,7 +3732,7 @@
         </is>
       </c>
       <c r="I36" t="n">
-        <v>0.6796762943267822</v>
+        <v>0.6911731958389282</v>
       </c>
       <c r="J36" t="n">
         <v>1</v>
@@ -3688,13 +3743,12 @@
           <t>Diagnosis / Impression:
 - No pleural effusion visible on the chest X-ray. [R1-IMAGE], [R2-IMAGE]
 Supporting Evidence:
-- The chest x-ray does not show any visible pleural effusion. [R1-IMAGE]
-- The chest X-ray does not show any visible pleural effusion. [R2-IMAGE]
-- Normal heart size and cardiomediastinal silhouette, which is consistent with no pleural effusion. [R1]
-- No focal airspace opacity, pleural effusion, or pneumothorax is observed on the chest X-ray. [R1]
+- The chest x-ray does not show any visible signs of pleural effusion. [R1-IMAGE]
+- The chest x-ray does not show any visible signs of pleural effusion. [R2-IMAGE]
+- The heart size and cardiomediastinal silhouette are normal, which is consistent with the absence of pleural effusion. [R1]
 Next Steps / Recommendations:
-- Clinical correlation recommended to assess the patient's symptoms and medical history. [Rx]
-- Follow-up imaging if symptoms persist or if the clinical correlation is inconclusive. [Rx]</t>
+- Clinical correlation recommended to rule out other causes of respiratory symptoms. [Rx]
+- Follow-up imaging if symptoms persist, but pleural effusion is unlikely given the current chest X-ray findings. [Rx]</t>
         </is>
       </c>
       <c r="M36" t="inlineStr"/>
@@ -3708,16 +3762,16 @@
         <v>1</v>
       </c>
       <c r="Q36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R36" t="n">
         <v>0.646</v>
       </c>
       <c r="S36" t="n">
-        <v>0.7323028882980347</v>
+        <v>0.7929519587516785</v>
       </c>
       <c r="T36" t="n">
-        <v>0.6891514441490174</v>
+        <v>0.7194759793758392</v>
       </c>
       <c r="U36" t="inlineStr">
         <is>
@@ -3753,7 +3807,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E37" t="n">
         <v>1</v>
@@ -3800,7 +3854,7 @@
         <v>1</v>
       </c>
       <c r="Q37" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R37" t="n">
         <v>0.672</v>
@@ -3845,7 +3899,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>0.75</v>
       </c>
       <c r="E38" t="n">
         <v>1</v>
@@ -3892,7 +3946,7 @@
         <v>1</v>
       </c>
       <c r="Q38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R38" t="n">
         <v>0.475</v>
@@ -3937,7 +3991,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="E39" t="n">
         <v>1</v>
@@ -3946,7 +4000,7 @@
         <v>1</v>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>0.714</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -3954,7 +4008,7 @@
         </is>
       </c>
       <c r="I39" t="n">
-        <v>0.8658748865127563</v>
+        <v>0.7861149907112122</v>
       </c>
       <c r="J39" t="n">
         <v>1</v>
@@ -3963,15 +4017,15 @@
       <c r="L39" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- No significant pathologies detected above threshold. [R1], [R2]
+- No significant pathologies detected above threshold. [R1]
 Supporting Evidence:
 - Lungs are clear. [R1]
 - No pneumothorax or pleural effusion detected. [R1]
 - Heart and mediastinum are within normal limits. [R1]
 - Bony structures are intact. [R1]
 Next Steps / Recommendations:
-- Clinical correlation recommended to further evaluate the patient's respiratory symptoms. [Rx]
-- Follow-up imaging if symptoms persist, as the current findings do not explain the patient's shortness of breath. [Rx]</t>
+- Clinical correlation recommended to further evaluate the patient's symptoms. [Rx]
+- Follow-up imaging if symptoms persist, but no immediate indication for further X-ray. [Rx]</t>
         </is>
       </c>
       <c r="M39" t="inlineStr"/>
@@ -3985,16 +4039,16 @@
         <v>1</v>
       </c>
       <c r="Q39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R39" t="n">
         <v>0.6</v>
       </c>
       <c r="S39" t="n">
-        <v>0.9597624659538269</v>
+        <v>0.8214344972133636</v>
       </c>
       <c r="T39" t="n">
-        <v>0.7798812329769134</v>
+        <v>0.7107172486066817</v>
       </c>
       <c r="U39" t="inlineStr">
         <is>
@@ -4030,7 +4084,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E40" t="n">
         <v>1</v>
@@ -4039,7 +4093,7 @@
         <v>1</v>
       </c>
       <c r="G40" t="n">
-        <v>0.714</v>
+        <v>0.5</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -4047,7 +4101,7 @@
         </is>
       </c>
       <c r="I40" t="n">
-        <v>0.5847504734992981</v>
+        <v>0.568744421005249</v>
       </c>
       <c r="J40" t="n">
         <v>1</v>
@@ -4056,15 +4110,14 @@
       <c r="L40" t="inlineStr">
         <is>
           <t>Diagnosis / Impression:
-- Insufficient evidence to indicate heart enlargement. [R1], [R2]
+- Insufficient evidence to confirm or rule out heart enlargement. [R1], [R2]
 Supporting Evidence:
-- The chest X-ray does not show any signs of heart enlargement. [R1-IMAGE]
-- The chest X-ray does not show any signs of heart enlargement. [R2-IMAGE]
-- The heart and mediastinum are normal on the chest X-ray. [R1]
-- Both lungs are clear and expanded on the chest X-ray. [R1]
+- The chest X-ray does not show any signs of heart enlargement. [R1-IMAGE], [R2-IMAGE]
+- A chest X-ray is not the most definitive imaging modality for assessing heart size, as it may not always provide clear visualization of the heart's structure. [R1-IMAGE]
+- Both lungs are clear and expanded, and the heart and mediastinum appear normal on the chest X-ray. [R1]
 Next Steps / Recommendations:
-- Clinical correlation recommended to further evaluate the patient's symptoms. [Rx]
-- Follow-up imaging if symptoms persist, but based on current evidence, it is not indicated. [Rx]</t>
+- Clinical correlation with other diagnostic modalities (e.g., echocardiogram, electrocardiogram) is recommended to further assess heart size and function. [Rx]
+- Follow-up imaging with a more definitive modality (e.g., echocardiogram) if symptoms persist or if there is a high clinical suspicion of heart enlargement. [Rx]</t>
         </is>
       </c>
       <c r="M40" t="inlineStr"/>
@@ -4078,16 +4131,16 @@
         <v>1</v>
       </c>
       <c r="Q40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R40" t="n">
         <v>0.458</v>
       </c>
       <c r="S40" t="n">
-        <v>0.7610251420497894</v>
+        <v>0.6706233263015747</v>
       </c>
       <c r="T40" t="n">
-        <v>0.6095125710248948</v>
+        <v>0.5643116631507874</v>
       </c>
       <c r="U40" t="inlineStr">
         <is>
@@ -4096,7 +4149,7 @@
       </c>
       <c r="V40" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>RETRY</t>
         </is>
       </c>
       <c r="W40" t="n">

</xml_diff>